<commit_message>
Tải dataset MIRAGE, tạo data manifest
</commit_message>
<xml_diff>
--- a/source_registry/source_registry_v1.xlsx
+++ b/source_registry/source_registry_v1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\Tiểu luận chuyên ngành\source_registry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0D3FD9-7B24-4E58-8E3D-0416725BC8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{936FBD34-7072-43D2-B7E0-5F86988886D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <author>Claude</author>
   </authors>
   <commentList>
-    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{A46BE088-AA84-4AC4-8A2D-4F37BBE3BA53}">
       <text>
         <r>
           <rPr>
@@ -67,7 +67,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{2172655B-D822-4A0B-87C3-E9E38761C982}">
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{59C70F81-FC11-4EB3-80DF-0DA9A2B38B42}">
       <text>
         <r>
           <rPr>
@@ -81,7 +81,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{59C70F81-FC11-4EB3-80DF-0DA9A2B38B42}">
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{2172655B-D822-4A0B-87C3-E9E38761C982}">
       <text>
         <r>
           <rPr>
@@ -95,7 +95,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C7" authorId="0" shapeId="0" xr:uid="{A46BE088-AA84-4AC4-8A2D-4F37BBE3BA53}">
+    <comment ref="C7" authorId="0" shapeId="0" xr:uid="{324466BC-81D2-4A30-B9DA-0C1A03A038DD}">
       <text>
         <r>
           <rPr>
@@ -109,7 +109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{324466BC-81D2-4A30-B9DA-0C1A03A038DD}">
+    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -163,9 +163,6 @@
     <t>note</t>
   </si>
   <si>
-    <t>SRC-001</t>
-  </si>
-  <si>
     <t>Giáo trình Y học cổ truyền- Thư viện số Y dược Mekong</t>
   </si>
   <si>
@@ -181,42 +178,24 @@
     <t>2026-09-14</t>
   </si>
   <si>
-    <t>SRC-002</t>
-  </si>
-  <si>
     <t>Sổ tay thuốc nam chữa bệnh tuyến cơ sở- Viện YHCT Quân đội</t>
   </si>
   <si>
     <t>Cao</t>
   </si>
   <si>
-    <t>SRC-003</t>
-  </si>
-  <si>
     <t>Phòng và chữa bệnh bằng cây thuốc nam- Viện YHCT Quân đội</t>
   </si>
   <si>
-    <t>SRC-004</t>
-  </si>
-  <si>
     <t>Bài giảng Y học cổ truyền tập 1- Khoa YHCT Đại học Y Hà Nội</t>
   </si>
   <si>
-    <t>SRC-005</t>
-  </si>
-  <si>
     <t>Bệnh học và điều trị đông y- Bộ Y tế</t>
   </si>
   <si>
-    <t>SRC-006</t>
-  </si>
-  <si>
     <t>Y lý Y học cổ truyền- Bộ Y tế</t>
   </si>
   <si>
-    <t>SRC-007</t>
-  </si>
-  <si>
     <t>Giáo trình Y học cổ truyền- Nhà xuất bản Đại học Quốc gia Hà Nội</t>
   </si>
   <si>
@@ -256,16 +235,37 @@
     <t>Công văn nhà nước</t>
   </si>
   <si>
-    <t>SRC-008</t>
-  </si>
-  <si>
-    <t>SRC-009</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://khoaduoc.pnt.edu.vn/vi/van-ban-phap-quy/quyet-dinh-so-3991-qd-byt-ve-viec-ban-hanh-tai-lieu-chuyen-mon-huong-dan-chan-doan-va-dieu-tri-benh-theo-y-hoc-co-truyen-ket-hop-y-hoc-co-truyen-voi-y-hoc-hien-dai-tap-ii  </t>
   </si>
   <si>
     <t xml:space="preserve">http://benhvienyhctlaocai.gov.vn/upload/21262/20220427/QD_5013_01_12_2020_Huong_dan_chan_doan_va_dieu_tri_yhct__yhct_ket_hop_yhhd_514b49e7dd.pdf   </t>
+  </si>
+  <si>
+    <t>SRC-01</t>
+  </si>
+  <si>
+    <t>SRC-02</t>
+  </si>
+  <si>
+    <t>SRC-03</t>
+  </si>
+  <si>
+    <t>SRC-04</t>
+  </si>
+  <si>
+    <t>SRC-07</t>
+  </si>
+  <si>
+    <t>SRC-05</t>
+  </si>
+  <si>
+    <t>SRC-06</t>
+  </si>
+  <si>
+    <t>SRC-08</t>
+  </si>
+  <si>
+    <t>SRC-09</t>
   </si>
 </sst>
 </file>
@@ -355,7 +355,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -364,20 +364,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -392,7 +391,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -701,15 +700,15 @@
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.109375" style="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.88671875" bestFit="1" customWidth="1"/>
   </cols>
@@ -750,312 +749,313 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>11</v>
+      <c r="A2" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="9">
+        <v>1</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="10" t="s">
+      <c r="J2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="H2" s="10">
-        <v>1</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>1</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>37</v>
+      <c r="I3" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>20</v>
+      <c r="A4" s="11" t="s">
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>40</v>
+        <v>18</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="10">
+      <c r="G4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="9">
         <v>1</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>37</v>
+      <c r="I4" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
-        <v>22</v>
+      <c r="A5" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="10">
+      <c r="G5" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="9">
         <v>1</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>37</v>
+      <c r="I5" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
-        <v>24</v>
+      <c r="A6" s="11" t="s">
+        <v>42</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>40</v>
+        <v>19</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="10">
+      <c r="G6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="9">
         <v>1</v>
       </c>
-      <c r="I6" s="10" t="s">
-        <v>37</v>
+      <c r="I6" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
-        <v>26</v>
+      <c r="A7" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>40</v>
+        <v>22</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="10">
+      <c r="G7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="9">
         <v>1</v>
       </c>
-      <c r="I7" s="10" t="s">
-        <v>37</v>
+      <c r="I7" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
-        <v>28</v>
+      <c r="A8" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>40</v>
+        <v>11</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="10">
+      <c r="H8" s="9">
         <v>1</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>37</v>
+      <c r="I8" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K8" s="3"/>
     </row>
     <row r="9" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
-        <v>42</v>
+      <c r="A9" s="11" t="s">
+        <v>44</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>41</v>
+        <v>31</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="10">
+      <c r="G9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="9">
         <v>1</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>37</v>
+      <c r="I9" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J9" s="7">
         <v>46279</v>
       </c>
-      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>41</v>
+      <c r="A10" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="10">
+      <c r="G10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="9">
         <v>1</v>
       </c>
-      <c r="I10" s="10" t="s">
-        <v>37</v>
+      <c r="I10" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="J10" s="7">
         <v>46279</v>
       </c>
-      <c r="K10" s="8"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K10">
+    <sortCondition ref="A1:A10"/>
+  </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{5E1C2811-F122-4D73-8714-7ACDB11A94D1}"/>
+    <hyperlink ref="D8" r:id="rId1" xr:uid="{5E1C2811-F122-4D73-8714-7ACDB11A94D1}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{4DA07BB0-28EA-4D10-A5C4-42D6E3F5C86A}"/>
     <hyperlink ref="D4" r:id="rId3" xr:uid="{8B3087E1-F874-4E05-AF55-3E382AB36982}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{DEBA09AF-6BA1-4838-B4BD-3AB68E024B19}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{890F6E67-A24F-457D-94A2-437325D24BF7}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{4ABEF015-2D2F-4935-B860-B828720A7383}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{88A3BF04-D5BF-4DCD-8985-DC907B5D9969}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{DEBA09AF-6BA1-4838-B4BD-3AB68E024B19}"/>
+    <hyperlink ref="D5" r:id="rId5" xr:uid="{890F6E67-A24F-457D-94A2-437325D24BF7}"/>
+    <hyperlink ref="D2" r:id="rId6" xr:uid="{4ABEF015-2D2F-4935-B860-B828720A7383}"/>
+    <hyperlink ref="D7" r:id="rId7" xr:uid="{88A3BF04-D5BF-4DCD-8985-DC907B5D9969}"/>
     <hyperlink ref="D9" r:id="rId8" xr:uid="{695BD57A-E170-4100-ABC7-FD44E9317514}"/>
     <hyperlink ref="D10" r:id="rId9" xr:uid="{63B1EDDD-BD6A-45A2-9FC7-EE2046431408}"/>
   </hyperlinks>

</xml_diff>